<commit_message>
Replace regex security scanner with Tree-sitter Java AST analyzer
</commit_message>
<xml_diff>
--- a/Milestone docs/Agile_Template_v0.1.xlsx
+++ b/Milestone docs/Agile_Template_v0.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI-Code-Review-Agent\Milestone docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D71788-C5BD-4AC9-BFB5-94FC6F0700B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD1C217-6A7F-4770-BE8D-82186B640F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories Plan" sheetId="1" r:id="rId1"/>

</xml_diff>